<commit_message>
Async media indexing: enqueue prepare/describe to a worker + status polling
- Add jobs table and backend/worker.py (DB-polled, one job at a time, stale-job recovery)
- Prepare/describe endpoints enqueue and return immediately; media serialize exposes job status/stage
- derive_status returns 'processing' while a job is active
- MediaTesting polls job status into the progress card and resumes on refresh
- Add media-worker component to .do/app.yaml; document local worker in README
- Tests for enqueue, processing status, and worker claim/success/error/reclaim

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/One Company - One Story (1).xlsx
+++ b/One Company - One Story (1).xlsx
@@ -725,7 +725,7 @@
     <t>Establishes that this is a real institution, not a bootcamp</t>
   </si>
   <si>
-    <t>Masters' Union University. Bill passed by the Government of Haryana. What that means and what it changes. Board of Governors — Kohli, Gambhir, Bansal. EFMD, AACSB, BGA, BSIS, NSDC. Rankings. Campus at DLF Cyberpark, Gurugram.</t>
+    <t>Masters' Union is becoming a university, following approval from the Government of Haryana. What that means and what it changes. Board of Governors — Kohli, Gambhir, Bansal. EFMD, AACSB, BGA, BSIS, NSDC. Rankings. Campus at DLF Cyberpark, Gurugram.</t>
   </si>
   <si>
     <t>Haryana bill; Prospectus p9–14; Brand Deck p11</t>
@@ -2543,7 +2543,7 @@
     <t>University status</t>
   </si>
   <si>
-    <t>Masters' Union University — bill passed by the Government of Haryana</t>
+    <t>Masters' Union is becoming a university, following approval from the Government of Haryana.</t>
   </si>
   <si>
     <t>Haryana state legislation</t>
@@ -2870,7 +2870,7 @@
     <t>Named founders and seasons — strongest format available.</t>
   </si>
   <si>
-    <t>Masters' Union University. The bill has been passed by the Government of Haryana. Exact permitted wording to be issued by Legal — LOCKED line, never improvised.</t>
+    <t>Masters' Union is becoming a university, following approval from the Government of Haryana. Exact permitted wording to be issued by Legal — LOCKED line, never improvised.</t>
   </si>
   <si>
     <t>Acceptance rate</t>

</xml_diff>